<commit_message>
Update scanner fundamentals and portfolio
</commit_message>
<xml_diff>
--- a/output/NSE_Portfolio_Recommendations.xlsx
+++ b/output/NSE_Portfolio_Recommendations.xlsx
@@ -549,77 +549,77 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IDEA</t>
+          <t>CORDSCABLE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14.11</v>
+        <v>225.8</v>
       </c>
       <c r="E2" t="n">
-        <v>11.55</v>
+        <v>187.35</v>
       </c>
       <c r="F2" t="n">
-        <v>22.11</v>
+        <v>20.52</v>
       </c>
       <c r="G2" t="n">
-        <v>12.8</v>
+        <v>216.6</v>
       </c>
       <c r="H2" t="n">
-        <v>10.23</v>
+        <v>4.25</v>
       </c>
       <c r="I2" t="n">
-        <v>64.90000000000001</v>
+        <v>61.49</v>
       </c>
       <c r="J2" t="n">
-        <v>2.12</v>
+        <v>4.15</v>
       </c>
       <c r="K2" t="n">
         <v>75</v>
       </c>
       <c r="L2" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="N2" t="n">
-        <v>14.11</v>
+        <v>225.8</v>
       </c>
       <c r="O2" t="n">
-        <v>7087</v>
+        <v>442</v>
       </c>
       <c r="P2" t="n">
         <v>100000</v>
       </c>
       <c r="Q2" t="n">
-        <v>99997.57000000001</v>
+        <v>99803.60000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>10</v>
+        <v>9.98</v>
       </c>
       <c r="S2" t="n">
-        <v>12.7</v>
+        <v>203.22</v>
       </c>
       <c r="T2" t="n">
-        <v>9999.76</v>
+        <v>9980.360000000001</v>
       </c>
       <c r="U2" t="n">
-        <v>17.07</v>
+        <v>273.22</v>
       </c>
       <c r="V2" t="n">
-        <v>20.98</v>
+        <v>21</v>
       </c>
       <c r="W2" t="n">
-        <v>20979.49</v>
+        <v>20958.76</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>MODERATE CONVICTION</t>
+          <t>HIGH CONVICTION</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -634,77 +634,77 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DICIND</t>
+          <t>CALSOFT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>575.5</v>
+        <v>24.6</v>
       </c>
       <c r="E3" t="n">
-        <v>514.6799999999999</v>
+        <v>17.32</v>
       </c>
       <c r="F3" t="n">
-        <v>11.82</v>
+        <v>42.01</v>
       </c>
       <c r="G3" t="n">
-        <v>570</v>
+        <v>21.42</v>
       </c>
       <c r="H3" t="n">
-        <v>0.96</v>
+        <v>14.85</v>
       </c>
       <c r="I3" t="n">
-        <v>69.12</v>
+        <v>65.59</v>
       </c>
       <c r="J3" t="n">
-        <v>17.84</v>
+        <v>1.98</v>
       </c>
       <c r="K3" t="n">
-        <v>75</v>
+        <v>72.5</v>
       </c>
       <c r="L3" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="M3" t="n">
-        <v>77</v>
+        <v>83.5</v>
       </c>
       <c r="N3" t="n">
-        <v>575.5</v>
+        <v>24.6</v>
       </c>
       <c r="O3" t="n">
-        <v>173</v>
+        <v>4065</v>
       </c>
       <c r="P3" t="n">
         <v>100000</v>
       </c>
       <c r="Q3" t="n">
-        <v>99561.5</v>
+        <v>99999</v>
       </c>
       <c r="R3" t="n">
-        <v>9.960000000000001</v>
+        <v>10</v>
       </c>
       <c r="S3" t="n">
-        <v>517.95</v>
+        <v>22.14</v>
       </c>
       <c r="T3" t="n">
-        <v>9956.15</v>
+        <v>9999.9</v>
       </c>
       <c r="U3" t="n">
-        <v>690.6</v>
+        <v>29.77</v>
       </c>
       <c r="V3" t="n">
-        <v>20</v>
+        <v>21.02</v>
       </c>
       <c r="W3" t="n">
-        <v>19912.3</v>
+        <v>21019.79</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>MODERATE CONVICTION</t>
+          <t>HIGH CONVICTION</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -719,73 +719,73 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KTKBANK</t>
+          <t>DICIND</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>309.65</v>
+        <v>575.5</v>
       </c>
       <c r="E4" t="n">
-        <v>232.49</v>
+        <v>514.6799999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>33.19</v>
+        <v>11.82</v>
       </c>
       <c r="G4" t="n">
-        <v>220.4</v>
+        <v>570</v>
       </c>
       <c r="H4" t="n">
-        <v>40.49</v>
+        <v>0.96</v>
       </c>
       <c r="I4" t="n">
-        <v>65.09999999999999</v>
+        <v>69.12</v>
       </c>
       <c r="J4" t="n">
-        <v>0.86</v>
+        <v>17.84</v>
       </c>
       <c r="K4" t="n">
-        <v>61.25</v>
+        <v>75</v>
       </c>
       <c r="L4" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="M4" t="n">
-        <v>76.75</v>
+        <v>77</v>
       </c>
       <c r="N4" t="n">
-        <v>309.65</v>
+        <v>575.5</v>
       </c>
       <c r="O4" t="n">
-        <v>322</v>
+        <v>173</v>
       </c>
       <c r="P4" t="n">
         <v>100000</v>
       </c>
       <c r="Q4" t="n">
-        <v>99707.3</v>
+        <v>99561.5</v>
       </c>
       <c r="R4" t="n">
-        <v>9.970000000000001</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="S4" t="n">
-        <v>278.68</v>
+        <v>517.95</v>
       </c>
       <c r="T4" t="n">
-        <v>9970.73</v>
+        <v>9956.15</v>
       </c>
       <c r="U4" t="n">
-        <v>365.39</v>
+        <v>690.6</v>
       </c>
       <c r="V4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="W4" t="n">
-        <v>17947.31</v>
+        <v>19912.3</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DCBBANK</t>
+          <t>KTKBANK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -813,64 +813,64 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>182.04</v>
+        <v>309.65</v>
       </c>
       <c r="E5" t="n">
-        <v>181.4</v>
+        <v>231.56</v>
       </c>
       <c r="F5" t="n">
-        <v>0.35</v>
+        <v>33.72</v>
       </c>
       <c r="G5" t="n">
-        <v>150.79</v>
+        <v>220.4</v>
       </c>
       <c r="H5" t="n">
-        <v>20.72</v>
+        <v>40.49</v>
       </c>
       <c r="I5" t="n">
-        <v>42.67</v>
+        <v>65.56</v>
       </c>
       <c r="J5" t="n">
-        <v>0.74</v>
+        <v>0.88</v>
       </c>
       <c r="K5" t="n">
-        <v>65</v>
+        <v>61.25</v>
       </c>
       <c r="L5" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="M5" t="n">
-        <v>75.8</v>
+        <v>76.75</v>
       </c>
       <c r="N5" t="n">
-        <v>182.04</v>
+        <v>309.65</v>
       </c>
       <c r="O5" t="n">
-        <v>549</v>
+        <v>322</v>
       </c>
       <c r="P5" t="n">
         <v>100000</v>
       </c>
       <c r="Q5" t="n">
-        <v>99939.96000000001</v>
+        <v>99707.3</v>
       </c>
       <c r="R5" t="n">
-        <v>9.99</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="S5" t="n">
-        <v>163.84</v>
+        <v>278.68</v>
       </c>
       <c r="T5" t="n">
-        <v>9994</v>
+        <v>9970.73</v>
       </c>
       <c r="U5" t="n">
-        <v>214.81</v>
+        <v>365.39</v>
       </c>
       <c r="V5" t="n">
         <v>18</v>
       </c>
       <c r="W5" t="n">
-        <v>17989.19</v>
+        <v>17947.31</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>RECOVERY WATCH</t>
+          <t>NOT A RECOVERY</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CALSOFT</t>
+          <t>DCBBANK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -898,64 +898,64 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24.6</v>
+        <v>182.04</v>
       </c>
       <c r="E6" t="n">
-        <v>17.36</v>
+        <v>181.4</v>
       </c>
       <c r="F6" t="n">
-        <v>41.72</v>
+        <v>0.35</v>
       </c>
       <c r="G6" t="n">
-        <v>21.42</v>
+        <v>150.79</v>
       </c>
       <c r="H6" t="n">
-        <v>14.85</v>
+        <v>20.72</v>
       </c>
       <c r="I6" t="n">
-        <v>66.54000000000001</v>
+        <v>42.67</v>
       </c>
       <c r="J6" t="n">
-        <v>1.91</v>
+        <v>0.74</v>
       </c>
       <c r="K6" t="n">
-        <v>72.5</v>
+        <v>65</v>
       </c>
       <c r="L6" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="M6" t="n">
-        <v>75.5</v>
+        <v>75.8</v>
       </c>
       <c r="N6" t="n">
-        <v>24.6</v>
+        <v>182.04</v>
       </c>
       <c r="O6" t="n">
-        <v>4065</v>
+        <v>549</v>
       </c>
       <c r="P6" t="n">
         <v>100000</v>
       </c>
       <c r="Q6" t="n">
-        <v>99999</v>
+        <v>99939.96000000001</v>
       </c>
       <c r="R6" t="n">
-        <v>10</v>
+        <v>9.99</v>
       </c>
       <c r="S6" t="n">
-        <v>22.14</v>
+        <v>163.84</v>
       </c>
       <c r="T6" t="n">
-        <v>9999.9</v>
+        <v>9994</v>
       </c>
       <c r="U6" t="n">
-        <v>29.77</v>
+        <v>214.81</v>
       </c>
       <c r="V6" t="n">
-        <v>21.02</v>
+        <v>18</v>
       </c>
       <c r="W6" t="n">
-        <v>21019.79</v>
+        <v>17989.19</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>NOT A RECOVERY</t>
+          <t>RECOVERY WATCH</t>
         </is>
       </c>
     </row>
@@ -986,10 +986,10 @@
         <v>351.3</v>
       </c>
       <c r="E7" t="n">
-        <v>289.05</v>
+        <v>287.84</v>
       </c>
       <c r="F7" t="n">
-        <v>21.54</v>
+        <v>22.05</v>
       </c>
       <c r="G7" t="n">
         <v>220</v>
@@ -998,10 +998,10 @@
         <v>59.68</v>
       </c>
       <c r="I7" t="n">
-        <v>52.36</v>
+        <v>53.46</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5</v>
+        <v>0.34</v>
       </c>
       <c r="K7" t="n">
         <v>57.5</v>
@@ -1241,10 +1241,10 @@
         <v>72.47</v>
       </c>
       <c r="E10" t="n">
-        <v>58.18</v>
+        <v>58.12</v>
       </c>
       <c r="F10" t="n">
-        <v>24.55</v>
+        <v>24.68</v>
       </c>
       <c r="G10" t="n">
         <v>68</v>
@@ -1253,10 +1253,10 @@
         <v>6.57</v>
       </c>
       <c r="I10" t="n">
-        <v>63.57</v>
+        <v>63.59</v>
       </c>
       <c r="J10" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="K10" t="n">
         <v>61.25</v>

</xml_diff>